<commit_message>
fix(pipeline): implement Inspection x8 multiplier rule for v1.4.0
- Applied x8 multiplier safely in CombinedEngineService
- Prevented manual override mutation
- Fixed all 71 unit tests in regression suite
- Validated UI and API bounds
</commit_message>
<xml_diff>
--- a/backend/tests/fixtures/excel1.xlsx
+++ b/backend/tests/fixtures/excel1.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Consolidated Report" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Consolidated Report" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>

</xml_diff>

<commit_message>
fix(backend): use valid_records count * 8 for inspection multiplier rule, update test assertions
</commit_message>
<xml_diff>
--- a/backend/tests/fixtures/excel1.xlsx
+++ b/backend/tests/fixtures/excel1.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Consolidated Report" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Consolidated Report" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>

</xml_diff>

<commit_message>
fix(calc): correctly apply 8x multiplier to valid inspection days, update API schema for frontend transparency
</commit_message>
<xml_diff>
--- a/backend/tests/fixtures/excel1.xlsx
+++ b/backend/tests/fixtures/excel1.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Consolidated Report" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Consolidated Report" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>

</xml_diff>